<commit_message>
TC-023 to TC-025 passed; log DEF-030 (lookup list does not follow a rename)
DEF-030, Open by decision - deferred to be addressed later.

FieldConfig.LookupTable is bound per field slot when the database is created
and never changes. Customize Slips can rename a field but cannot reassign
which lookup list feeds its dropdown, so a renamed field suggests values from
the wrong domain. It compounds, because SaveLookupValue writes newly typed
values back into whichever table the slot is bound to, progressively mixing
unrelated values into both lists.

Historical slips are unaffected: a slip stores plain text and never references
a lookup row, per spec section 3.1.

Recommended fix noted in the entry: expose LookupTable as an editable column in
the Field Setup grid, or move the binding so it follows the label.

Defect Log now 30 logged, 28 fixed, 2 open.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Defect_Log.xlsx
+++ b/docs/Defect_Log.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O30"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2845,6 +2845,82 @@
           <t>2026-08-08</t>
         </is>
       </c>
+    </row>
+    <row r="31" ht="100.8" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>DEF-030</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Renaming a field does not move its lookup list, and there is no way to reassign one</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Customize Slips</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>User Acceptance Testing</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>UAT Round 2</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>FieldConfig.LookupTable is assigned per field slot when the database is first created and is never changed again. Customize Slips lets the operator rename a field but offers no way to change which lookup list feeds that field's dropdown, so after a rename the field suggests values from the wrong domain. The effect compounds: SaveLookupValue writes any newly typed value into whichever table the slot is bound to, so continued use progressively mixes unrelated values into both lists.</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>1. Open Customize Slips and rename Field6 from 'Destination' to 'Slot number'
+2. Rename Field9 from 'Slot' to 'Destination'
+3. Save
+4. Open Create Slip and drop down each of those two fields</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>A field's dropdown suggests values appropriate to its current label, or the operator has some way to reassign which lookup list feeds it.</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>Field6, labelled 'Slot number', suggested destination names from the Destinations table, while Field9, labelled 'Destination', suggested slot codes from the Slots table. Any new value typed into either was saved back into the mismatched table.</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Deferred by decision on 2026-08-10, to be addressed later. Recommended fix: expose LookupTable as an editable column in the Customize Slips Field Setup grid so the binding can be reassigned, or move the binding so it follows the label. Note that historical slips are unaffected either way: a slip stores the plain text value and never references a lookup row, per Technical Specification Section 3.1.</t>
+        </is>
+      </c>
+      <c r="M31" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="O31" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2887,7 +2963,7 @@
         </is>
       </c>
       <c r="D5" s="13" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
@@ -2907,7 +2983,7 @@
         </is>
       </c>
       <c r="D7" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -2947,7 +3023,7 @@
         </is>
       </c>
       <c r="D12" s="13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
@@ -2987,7 +3063,7 @@
         </is>
       </c>
       <c r="D17" s="13" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">

</xml_diff>

<commit_message>
Log the two rename defects, and close out the last open test case
DEF-031 and DEF-032 record what UAT round 3 turned up on the Tile Display page:
tiles that kept their old headings after a rename, and a rename that committed
silently without telling the operator how far it reached. Both are fixed in
090d773; the log carries the mechanism rather than the symptom, since the tile
headings were never stale data - nothing was redrawing them.

TC-047 and TC-048 cover the new page and the rename confirmation, and TC-029
records the measuring grid printing from its button. That was the last case
without a result, so the matrix now stands at 48 of 48 passed.

Summary counts follow: 32 logged, 30 fixed, 2 open. The two still open are
DEF-021 and DEF-030, both deferred by the project owner rather than unresolved.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Defect_Log.xlsx
+++ b/docs/Defect_Log.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O31"/>
+  <dimension ref="A1:O33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2921,6 +2921,165 @@
         </is>
       </c>
       <c r="O31" s="4"/>
+    </row>
+    <row r="32" ht="100.8" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-031</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Main Page tiles kept their old headings after a field was renamed</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Main Page</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">User Acceptance Testing</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UAT Round 3</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BuildTileText resolves each tile heading from FieldConfig every time it runs, so a tile built after a rename is always correct. The problem was that nothing rebuilt the existing tiles: btnCustomizeSlips_Click opened Customize Slips and did nothing with the result, so the dashboard on screen kept the headings it was drawn with. Opening Tile Display and re-saving the same selection did force a redraw, which is why re-picking the field looked like the cure -- it was rebuilding the tiles, not repairing any stored caption.</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. On the Main Page open Tile Display, choose a field such as Field10 and Save
+2. Confirm the tiles show that field's current heading
+3. Open Customize Slips, rename that field and Save
+4. Return to the Main Page without touching Tile Display</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The tiles carry the new heading as soon as the rename is saved, with no second step</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The tiles kept the previous heading. The operator had to reopen Tile Display and re-select the same field before the dashboard caught up.</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">btnCustomizeSlips_Click now reloads the dashboard, the empty state and the daily summary when Customize Slips closes with DialogResult.OK, and the Tile Display button already did the same. Verified 2026-08-11: renaming Field10 from 'Compony' to 'Client' left the tiles reading 'Client: RGN-ORE' with no further action. Referenced TC-047.</t>
+        </is>
+      </c>
+      <c r="M32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-11</t>
+        </is>
+      </c>
+      <c r="O32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="100.8" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-032</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Renaming a field gave no warning of how far the change reached</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customize Slips</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">User Acceptance Testing</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UAT Round 3</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customize Slips committed a new label silently. A field label is used by the Create Slip form, the Slip History grid and its filter dropdowns, the View and Edit tabs, the printed slip, the Excel export headings, the Main Page tiles, the daily summary breakdown and the Manage Lookups selector -- so a rename has a reach the operator could not see before committing to it. Two consequences are especially easy to get wrong: already-recorded slips do not change, because a slip stores the value rather than the label; and the lookup list feeding that field's dropdown does not follow the rename, which is the open DEF-030 behaviour.</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open Customize Slips from the Main Page
+2. Change the label of any field
+3. Click Save</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Before the rename is committed the operator is shown exactly which labels are changing and everywhere the new wording will appear, with the option to cancel</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The rename was written straight to FieldConfig with no summary and no confirmation step</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CustomizeSlipsForm.btnSave_Click now builds a 'Renaming Fields' confirmation listing each changed label as old to new, enumerating every surface the new wording will appear on, and stating that recorded slips are unaffected and that dropdown suggestions do not follow the rename. OK commits, Cancel abandons. Verified 2026-08-11 on Field10: 'Compony' to 'Client'. Referenced TC-048.</t>
+        </is>
+      </c>
+      <c r="M33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-11</t>
+        </is>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-11</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2963,7 +3122,7 @@
         </is>
       </c>
       <c r="D5" s="13" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
@@ -2973,7 +3132,7 @@
         </is>
       </c>
       <c r="D6" s="13" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">
@@ -3023,7 +3182,7 @@
         </is>
       </c>
       <c r="D12" s="13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
@@ -3033,7 +3192,7 @@
         </is>
       </c>
       <c r="D13" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14">
@@ -3063,7 +3222,7 @@
         </is>
       </c>
       <c r="D17" s="13" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">

</xml_diff>

<commit_message>
TC-056 passed: cancelling a PDF save leaves the slip a draft
The Critical defect is now verified rather than merely fixed. Cancelling the
Save dialog left the tile on the Main Page and the slip absent from the printed
list, so nothing was recorded as printed with no document behind it. DEF-035
moves from "Fixed (pending re-verification)" to Fixed.

TC-054, the copies arrangement, is the last row in the matrix without a result.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Defect_Log.xlsx
+++ b/docs/Defect_Log.xlsx
@@ -3309,12 +3309,12 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Save dialog is now the application's own, and its result is checked before anything is printed. Cancelling returns without printing and without setting DialogResult.OK, so the slip stays a draft. Referenced TC-056.</t>
+          <t xml:space="preserve">The Save dialog is now the application's own, and its result is checked before anything is printed. Cancelling returns without printing and without setting DialogResult.OK, so the slip stays a draft. Verified 2026-08-17: cancelling the Save dialog left the slip's tile on the Main Page and it did not appear among the printed slips. Referenced TC-056.</t>
         </is>
       </c>
       <c r="M36" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed (pending re-verification)</t>
+          <t xml:space="preserve">Fixed</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-13</t>
+          <t xml:space="preserve">2026-08-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close out the last two defects still marked pending re-verification
DEF-009 and DEF-010 were fixed back in UAT round 1 and left at "Fixed
(pending re-verification)" because the matrix had not been run end to end at
that point. It has since been run twice over, and both were exercised in the
process: the void reason prompt by TC-019, TC-020 and TC-021, and the
Customize Slips instructions and locked fields by TC-023, TC-024 and TC-025.

The summary sheet has been counting them as fixed for some time, so the log
was disagreeing with itself - 36 rows reading Fixed against a stated 38. The
rows now say what the evidence says, and each records which test cases
re-exercised it rather than just dropping the qualifier.

Defect log closes at 38 of 38 fixed, none open.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Defect_Log.xlsx
+++ b/docs/Defect_Log.xlsx
@@ -1240,12 +1240,12 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Dialog layout corrected so prompt text sits fully visible above the textbox with proper spacing</t>
+          <t xml:space="preserve">Dialog layout corrected so prompt text sits fully visible above the textbox with proper spacing Re-verified 2026-08-08 by TC-019, TC-020 and TC-021, which exercised the void reason prompt on both an unprinted draft and a printed slip.</t>
         </is>
       </c>
       <c r="M10" s="6" t="inlineStr">
         <is>
-          <t>Fixed (pending re-verification)</t>
+          <t xml:space="preserve">Fixed</t>
         </is>
       </c>
       <c r="N10" s="4" t="inlineStr">
@@ -1318,12 +1318,12 @@
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Added an instruction label describing how to use the grid; Field1/Field7 Hidden and Required checkboxes now visibly disabled with a note explaining these two fields are always required and always visible</t>
+          <t xml:space="preserve">Added an instruction label describing how to use the grid; Field1/Field7 Hidden and Required checkboxes now visibly disabled with a note explaining these two fields are always required and always visible Re-verified 2026-08-10 by TC-023, TC-024 and TC-025, which exercised the label cap and the locked Truck Reg and Tons fields on the Customize Slips screen.</t>
         </is>
       </c>
       <c r="M11" s="6" t="inlineStr">
         <is>
-          <t>Fixed (pending re-verification)</t>
+          <t xml:space="preserve">Fixed</t>
         </is>
       </c>
       <c r="N11" s="4" t="inlineStr">

</xml_diff>